<commit_message>
Initial commit: AI Anomaly Watcher setup
</commit_message>
<xml_diff>
--- a/data/business_metrics.xlsx
+++ b/data/business_metrics.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4882.041430931009</v>
+        <v>4936.948237487465</v>
       </c>
       <c r="C2" t="n">
-        <v>100.7865719239505</v>
+        <v>100.40171235518</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02934574120329208</v>
+        <v>0.03058090752405993</v>
       </c>
       <c r="E2" t="n">
-        <v>3293.96563233387</v>
+        <v>3140.586651624125</v>
       </c>
       <c r="F2" t="n">
-        <v>1216.109184837661</v>
+        <v>1452.866740620603</v>
       </c>
     </row>
     <row r="3">
@@ -477,19 +477,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5140.390845988524</v>
+        <v>5137.072178271002</v>
       </c>
       <c r="C3" t="n">
-        <v>103.4841179170918</v>
+        <v>97.53697736016487</v>
       </c>
       <c r="D3" t="n">
-        <v>0.03340709051790095</v>
+        <v>0.03283021622320651</v>
       </c>
       <c r="E3" t="n">
-        <v>3402.309183493882</v>
+        <v>3146.263648461852</v>
       </c>
       <c r="F3" t="n">
-        <v>1296.832177329294</v>
+        <v>1587.948922728602</v>
       </c>
     </row>
     <row r="4">
@@ -499,19 +499,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4938.863452123333</v>
+        <v>5063.755129487968</v>
       </c>
       <c r="C4" t="n">
-        <v>99.84118529254464</v>
+        <v>94.67987192215432</v>
       </c>
       <c r="D4" t="n">
-        <v>0.03166516646359472</v>
+        <v>0.02881977025819872</v>
       </c>
       <c r="E4" t="n">
-        <v>3373.560859470951</v>
+        <v>3146.931307036888</v>
       </c>
       <c r="F4" t="n">
-        <v>1543.172405959574</v>
+        <v>1583.287094555287</v>
       </c>
     </row>
     <row r="5">
@@ -521,19 +521,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5636.871348611476</v>
+        <v>4955.488263877246</v>
       </c>
       <c r="C5" t="n">
-        <v>103.5425968958394</v>
+        <v>100.3505869201235</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03188790222546287</v>
+        <v>0.0282738930108435</v>
       </c>
       <c r="E5" t="n">
-        <v>3277.947008512906</v>
+        <v>3367.386970606463</v>
       </c>
       <c r="F5" t="n">
-        <v>1472.707665999728</v>
+        <v>1633.005447524986</v>
       </c>
     </row>
     <row r="6">
@@ -543,19 +543,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4994.544279282261</v>
+        <v>4973.959143662645</v>
       </c>
       <c r="C6" t="n">
-        <v>98.9673839756089</v>
+        <v>97.2615793032614</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02945000814027768</v>
+        <v>0.02661656842034099</v>
       </c>
       <c r="E6" t="n">
-        <v>3465.134694861247</v>
+        <v>3196.464729774803</v>
       </c>
       <c r="F6" t="n">
-        <v>1622.190179378839</v>
+        <v>1631.802366797934</v>
       </c>
     </row>
     <row r="7">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5097.31713499278</v>
+        <v>5349.591876579551</v>
       </c>
       <c r="C7" t="n">
-        <v>101.3333691897016</v>
+        <v>102.067150655237</v>
       </c>
       <c r="D7" t="n">
-        <v>0.02994599631674949</v>
+        <v>0.03111710549488879</v>
       </c>
       <c r="E7" t="n">
-        <v>3435.819320458345</v>
+        <v>3173.973696351985</v>
       </c>
       <c r="F7" t="n">
-        <v>1477.452710125291</v>
+        <v>1445.847123473791</v>
       </c>
     </row>
     <row r="8">
@@ -587,19 +587,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4981.370400923291</v>
+        <v>5123.573493499802</v>
       </c>
       <c r="C8" t="n">
-        <v>108.2929662716769</v>
+        <v>108.001482643633</v>
       </c>
       <c r="D8" t="n">
-        <v>0.03125963258599584</v>
+        <v>0.02906469625428689</v>
       </c>
       <c r="E8" t="n">
-        <v>3368.275884661529</v>
+        <v>3265.669307158302</v>
       </c>
       <c r="F8" t="n">
-        <v>1430.056652104681</v>
+        <v>1612.922497168291</v>
       </c>
     </row>
     <row r="9">
@@ -609,19 +609,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5019.97116643968</v>
+        <v>4866.478203029412</v>
       </c>
       <c r="C9" t="n">
-        <v>105.3174113788157</v>
+        <v>98.73284127989082</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02814835626597733</v>
+        <v>0.02855278941457597</v>
       </c>
       <c r="E9" t="n">
-        <v>3417.807415723925</v>
+        <v>3311.646099681775</v>
       </c>
       <c r="F9" t="n">
-        <v>1661.263143015347</v>
+        <v>1556.681960619877</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5043.102371253264</v>
+        <v>4895.206689271001</v>
       </c>
       <c r="C10" t="n">
-        <v>100.1499458079568</v>
+        <v>95.38849125094185</v>
       </c>
       <c r="D10" t="n">
-        <v>0.03214462263314635</v>
+        <v>0.02989593282300851</v>
       </c>
       <c r="E10" t="n">
-        <v>3176.494313292237</v>
+        <v>3465.614962186242</v>
       </c>
       <c r="F10" t="n">
-        <v>1586.228820138974</v>
+        <v>1463.497715758954</v>
       </c>
     </row>
     <row r="11">
@@ -653,19 +653,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5161.024639639815</v>
+        <v>5043.272055454897</v>
       </c>
       <c r="C11" t="n">
-        <v>99.04638340447028</v>
+        <v>96.96763465469431</v>
       </c>
       <c r="D11" t="n">
-        <v>0.03051907183021796</v>
+        <v>0.02788472917827651</v>
       </c>
       <c r="E11" t="n">
-        <v>3048.602206895526</v>
+        <v>3342.683295314406</v>
       </c>
       <c r="F11" t="n">
-        <v>1622.881484010529</v>
+        <v>1465.397930500824</v>
       </c>
     </row>
     <row r="12">
@@ -675,19 +675,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4888.720870282823</v>
+        <v>4871.580870285258</v>
       </c>
       <c r="C12" t="n">
-        <v>108.4481260715705</v>
+        <v>98.09817018907951</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02926673659835366</v>
+        <v>0.02930044958066395</v>
       </c>
       <c r="E12" t="n">
-        <v>3294.062083761618</v>
+        <v>3303.237353631796</v>
       </c>
       <c r="F12" t="n">
-        <v>1629.007519909448</v>
+        <v>1401.753159361112</v>
       </c>
     </row>
     <row r="13">
@@ -697,19 +697,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4618.480958200137</v>
+        <v>5230.956725102155</v>
       </c>
       <c r="C13" t="n">
-        <v>115.4769958150304</v>
+        <v>103.7875218161051</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02922620072928986</v>
+        <v>0.02574660408343169</v>
       </c>
       <c r="E13" t="n">
-        <v>3236.131870431715</v>
+        <v>3278.576295740528</v>
       </c>
       <c r="F13" t="n">
-        <v>1433.858526506225</v>
+        <v>1334.36265684154</v>
       </c>
     </row>
     <row r="14">
@@ -719,19 +719,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4758.782827363772</v>
+        <v>5106.832478770995</v>
       </c>
       <c r="C14" t="n">
-        <v>106.2144648437946</v>
+        <v>88.88052065775412</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02606880975061166</v>
+        <v>0.02868648343003378</v>
       </c>
       <c r="E14" t="n">
-        <v>3144.812470262159</v>
+        <v>3247.790576195971</v>
       </c>
       <c r="F14" t="n">
-        <v>1500.886224292721</v>
+        <v>1483.607298571545</v>
       </c>
     </row>
     <row r="15">
@@ -741,19 +741,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5324.669987111328</v>
+        <v>5120.629076344378</v>
       </c>
       <c r="C15" t="n">
-        <v>94.04440626364195</v>
+        <v>106.1954893435912</v>
       </c>
       <c r="D15" t="n">
-        <v>0.03126632461338787</v>
+        <v>0.02840170609250186</v>
       </c>
       <c r="E15" t="n">
-        <v>3512.50717964979</v>
+        <v>3206.765881929371</v>
       </c>
       <c r="F15" t="n">
-        <v>1637.851923795925</v>
+        <v>1553.914322866371</v>
       </c>
     </row>
     <row r="16">
@@ -763,19 +763,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5275.002560564273</v>
+        <v>5151.401375429332</v>
       </c>
       <c r="C16" t="n">
-        <v>105.8404919483021</v>
+        <v>97.32407527681497</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02946029758353736</v>
+        <v>0.02968176704942901</v>
       </c>
       <c r="E16" t="n">
-        <v>3331.842779094869</v>
+        <v>3109.689242791942</v>
       </c>
       <c r="F16" t="n">
-        <v>1579.440482237574</v>
+        <v>1425.784810911248</v>
       </c>
     </row>
     <row r="17">
@@ -785,19 +785,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4562.566491477808</v>
+        <v>4957.995116872267</v>
       </c>
       <c r="C17" t="n">
-        <v>99.50462207732978</v>
+        <v>102.1258568840819</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0295448217022071</v>
+        <v>0.03421502859668733</v>
       </c>
       <c r="E17" t="n">
-        <v>3387.675552788402</v>
+        <v>3006.364964698432</v>
       </c>
       <c r="F17" t="n">
-        <v>1686.422469645188</v>
+        <v>1647.424732470695</v>
       </c>
     </row>
     <row r="18">
@@ -807,19 +807,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4896.596972266988</v>
+        <v>4923.93759513542</v>
       </c>
       <c r="C18" t="n">
-        <v>101.1426676906019</v>
+        <v>100.2304428884999</v>
       </c>
       <c r="D18" t="n">
-        <v>0.03197353260956171</v>
+        <v>0.03059815033022351</v>
       </c>
       <c r="E18" t="n">
-        <v>3247.607399568164</v>
+        <v>3030.655293792699</v>
       </c>
       <c r="F18" t="n">
-        <v>1540.962248776205</v>
+        <v>1540.251707128378</v>
       </c>
     </row>
     <row r="19">
@@ -829,19 +829,19 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>5395.300809472595</v>
+        <v>5081.613318346472</v>
       </c>
       <c r="C19" t="n">
-        <v>100.6980882289024</v>
+        <v>99.66776129259217</v>
       </c>
       <c r="D19" t="n">
-        <v>0.03243012016036801</v>
+        <v>0.02775117176825848</v>
       </c>
       <c r="E19" t="n">
-        <v>3254.724407350504</v>
+        <v>3621.560996655247</v>
       </c>
       <c r="F19" t="n">
-        <v>1450.679658338253</v>
+        <v>1359.819241955551</v>
       </c>
     </row>
     <row r="20">
@@ -851,19 +851,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4798.774175304316</v>
+        <v>5091.551900694996</v>
       </c>
       <c r="C20" t="n">
-        <v>100.5689157455204</v>
+        <v>97.26762437658877</v>
       </c>
       <c r="D20" t="n">
-        <v>0.02803162335754653</v>
+        <v>0.02869875708392802</v>
       </c>
       <c r="E20" t="n">
-        <v>3102.865095482172</v>
+        <v>3464.905541170219</v>
       </c>
       <c r="F20" t="n">
-        <v>1392.095565357478</v>
+        <v>1411.106444006102</v>
       </c>
     </row>
     <row r="21">
@@ -873,19 +873,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5103.879378878702</v>
+        <v>4920.79055060734</v>
       </c>
       <c r="C21" t="n">
-        <v>103.002870095116</v>
+        <v>93.51510743595747</v>
       </c>
       <c r="D21" t="n">
-        <v>0.02873636496928657</v>
+        <v>0.02931519732236867</v>
       </c>
       <c r="E21" t="n">
-        <v>3310.699502747352</v>
+        <v>3067.372806469769</v>
       </c>
       <c r="F21" t="n">
-        <v>1394.185102656236</v>
+        <v>1364.242810337403</v>
       </c>
     </row>
     <row r="22">
@@ -895,19 +895,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4853.259382451182</v>
+        <v>4689.46374747752</v>
       </c>
       <c r="C22" t="n">
-        <v>91.57672645864429</v>
+        <v>103.6320341826423</v>
       </c>
       <c r="D22" t="n">
-        <v>0.03005063752426487</v>
+        <v>0.03170247236290533</v>
       </c>
       <c r="E22" t="n">
-        <v>3417.328087782137</v>
+        <v>3356.840197225011</v>
       </c>
       <c r="F22" t="n">
-        <v>1576.362950856287</v>
+        <v>1323.229208363995</v>
       </c>
     </row>
     <row r="23">
@@ -917,19 +917,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4830.388193667967</v>
+        <v>4565.199817534301</v>
       </c>
       <c r="C23" t="n">
-        <v>93.59739463970379</v>
+        <v>97.18696288016002</v>
       </c>
       <c r="D23" t="n">
-        <v>0.02699823821482682</v>
+        <v>0.03066103919391532</v>
       </c>
       <c r="E23" t="n">
-        <v>3463.855941333936</v>
+        <v>3197.715473475916</v>
       </c>
       <c r="F23" t="n">
-        <v>1535.556198250451</v>
+        <v>1586.884037725622</v>
       </c>
     </row>
     <row r="24">
@@ -939,19 +939,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5113.948062816105</v>
+        <v>5089.629829060346</v>
       </c>
       <c r="C24" t="n">
-        <v>112.3318183491614</v>
+        <v>101.8207010738498</v>
       </c>
       <c r="D24" t="n">
-        <v>0.03036129224566369</v>
+        <v>0.02709297750149641</v>
       </c>
       <c r="E24" t="n">
-        <v>3446.7549416611</v>
+        <v>3289.432721070222</v>
       </c>
       <c r="F24" t="n">
-        <v>1717.883698429986</v>
+        <v>1410.372795089683</v>
       </c>
     </row>
     <row r="25">
@@ -961,19 +961,19 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>4926.527154333613</v>
+        <v>5301.065824525108</v>
       </c>
       <c r="C25" t="n">
-        <v>97.57789820227073</v>
+        <v>93.16090655934575</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0301530813605655</v>
+        <v>0.0287296519459182</v>
       </c>
       <c r="E25" t="n">
-        <v>3415.954360351826</v>
+        <v>3205.430452831392</v>
       </c>
       <c r="F25" t="n">
-        <v>1395.208384782612</v>
+        <v>1391.928991527981</v>
       </c>
     </row>
     <row r="26">
@@ -983,19 +983,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4687.477147441797</v>
+        <v>4822.900169928671</v>
       </c>
       <c r="C26" t="n">
-        <v>98.90493566957882</v>
+        <v>101.3807370078786</v>
       </c>
       <c r="D26" t="n">
-        <v>0.02958951383977745</v>
+        <v>0.03121881171398465</v>
       </c>
       <c r="E26" t="n">
-        <v>3182.766352749397</v>
+        <v>3185.824033872721</v>
       </c>
       <c r="F26" t="n">
-        <v>1499.734034962195</v>
+        <v>1479.746148734058</v>
       </c>
     </row>
     <row r="27">
@@ -1005,19 +1005,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4979.032667323308</v>
+        <v>4928.524539810895</v>
       </c>
       <c r="C27" t="n">
-        <v>94.50036451586958</v>
+        <v>93.01942303372176</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0290095027185581</v>
+        <v>0.02586526542538499</v>
       </c>
       <c r="E27" t="n">
-        <v>3321.482946626025</v>
+        <v>3092.482847536052</v>
       </c>
       <c r="F27" t="n">
-        <v>1392.06894079851</v>
+        <v>1600.414080533577</v>
       </c>
     </row>
     <row r="28">
@@ -1027,19 +1027,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>5018.757701737506</v>
+        <v>5050.838142435307</v>
       </c>
       <c r="C28" t="n">
-        <v>104.5118773255204</v>
+        <v>95.19264942094036</v>
       </c>
       <c r="D28" t="n">
-        <v>0.03039682369639562</v>
+        <v>0.03462265572037149</v>
       </c>
       <c r="E28" t="n">
-        <v>3535.607240969835</v>
+        <v>3315.314104829344</v>
       </c>
       <c r="F28" t="n">
-        <v>1413.081902762815</v>
+        <v>1612.461061058188</v>
       </c>
     </row>
     <row r="29">
@@ -1049,19 +1049,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4832.943568316706</v>
+        <v>4581.383283534508</v>
       </c>
       <c r="C29" t="n">
-        <v>100.5529614919285</v>
+        <v>89.42639283480428</v>
       </c>
       <c r="D29" t="n">
-        <v>0.03072638504141951</v>
+        <v>0.03082312821211091</v>
       </c>
       <c r="E29" t="n">
-        <v>3313.297676654564</v>
+        <v>3614.32509735273</v>
       </c>
       <c r="F29" t="n">
-        <v>1476.62331405795</v>
+        <v>1472.369407506468</v>
       </c>
     </row>
     <row r="30">
@@ -1071,19 +1071,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>4930.235197382079</v>
+        <v>4608.08316241237</v>
       </c>
       <c r="C30" t="n">
-        <v>98.38296962002534</v>
+        <v>100.3255670839187</v>
       </c>
       <c r="D30" t="n">
-        <v>0.02970625369733816</v>
+        <v>0.03371146306250898</v>
       </c>
       <c r="E30" t="n">
-        <v>3256.236662019041</v>
+        <v>2972.720529814569</v>
       </c>
       <c r="F30" t="n">
-        <v>1353.374575740655</v>
+        <v>1398.331254799586</v>
       </c>
     </row>
     <row r="31">

</xml_diff>